<commit_message>
feat: Suite movil completa con 35 campos, auto-calculo de criticidad, edicion, eliminacion y configuracion para Render
</commit_message>
<xml_diff>
--- a/plantillas/plantilla_muebleria.xlsx
+++ b/plantillas/plantilla_muebleria.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Desktop\CMMS_GAMLP\plantillas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C75C59FF-0C92-400D-A2E0-474AF79F0AEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4852CBA7-D2FA-4769-9F31-82F91D5995E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{D3B5DAA1-68B9-4EE4-905B-A41A732D50B3}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>SECTOR_ACTUAL</t>
   </si>
@@ -81,7 +81,10 @@
     <t>UBICACION</t>
   </si>
   <si>
-    <t>FECHA_INCORPORACION</t>
+    <t>ESTADO</t>
+  </si>
+  <si>
+    <t>MARCA</t>
   </si>
 </sst>
 </file>
@@ -468,10 +471,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DFE3A508-2887-45DB-97C9-0CF971D91181}">
-  <dimension ref="A1:R1"/>
+  <dimension ref="A1:S1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:19" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -500,30 +503,33 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="K1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="M1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="3" t="s">
+      <c r="Q1" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="3" t="s">
+      <c r="R1" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="3" t="s">
+      <c r="S1" s="3" t="s">
         <v>17</v>
       </c>
     </row>

</xml_diff>